<commit_message>
Update example_scenario.xlsx to include parameters and sheet for stock lifetime overrides
</commit_message>
<xml_diff>
--- a/src/aiphoria/data/example_scenario.xlsx
+++ b/src/aiphoria/data/example_scenario.xlsx
@@ -1,25 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\PythonProjects\aiphoria\src\aiphoria\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{999E48CA-8F24-43CA-BCCB-1C08627B4779}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FF67D8E-CB75-437F-A89D-3471ED78FF46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1000A452-A98F-45C1-B843-91F7F67E097C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{1000A452-A98F-45C1-B843-91F7F67E097C}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="11" r:id="rId1"/>
     <sheet name="Processes" sheetId="6" r:id="rId2"/>
     <sheet name="Flows" sheetId="1" r:id="rId3"/>
-    <sheet name="Process positions" sheetId="14" r:id="rId4"/>
-    <sheet name="Scenarios" sheetId="12" r:id="rId5"/>
-    <sheet name="Colors" sheetId="13" r:id="rId6"/>
-    <sheet name="Data validation parameters" sheetId="9" r:id="rId7"/>
+    <sheet name="Stock lifetime overrides" sheetId="15" r:id="rId4"/>
+    <sheet name="Process positions" sheetId="14" r:id="rId5"/>
+    <sheet name="Scenarios" sheetId="12" r:id="rId6"/>
+    <sheet name="Colors" sheetId="13" r:id="rId7"/>
+    <sheet name="Data validation parameters" sheetId="9" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Flows!$A$3:$P$13</definedName>
@@ -48,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="240">
   <si>
     <t>Years</t>
   </si>
@@ -254,15 +255,9 @@
     <t>skip_num_rows_flows</t>
   </si>
   <si>
-    <t>Sheet name that contains data for Processes, e.g. (Processes)</t>
-  </si>
-  <si>
     <t>Number of rows to skip when reading data for Processes (e.g. 2). NOTE: Header row must be the first row to read!</t>
   </si>
   <si>
-    <t>Sheet name that contains data for Flows, (e.g. Flows)</t>
-  </si>
-  <si>
     <t>start_year</t>
   </si>
   <si>
@@ -360,9 +355,6 @@
   </si>
   <si>
     <t>Scenarios</t>
-  </si>
-  <si>
-    <t>Sheet name that contains scenarios (flow variations)</t>
   </si>
   <si>
     <t>create_network_graphs</t>
@@ -538,9 +530,6 @@
     <t>Colors</t>
   </si>
   <si>
-    <t>Sheet name that contains data for transformation stage colors (e.g. Colors)</t>
-  </si>
-  <si>
     <t>#808080</t>
   </si>
   <si>
@@ -715,9 +704,6 @@
     <t>Process positions</t>
   </si>
   <si>
-    <t>Sheet name that contains data for process positions in normalized format (position data in range [0,1])</t>
-  </si>
-  <si>
     <t>Industrial_roundwood:FI</t>
   </si>
   <si>
@@ -755,6 +741,78 @@
   </si>
   <si>
     <t>Include scenario metadata (currently filename) to Sankey visualization</t>
+  </si>
+  <si>
+    <t>number</t>
+  </si>
+  <si>
+    <t>This column is ignored (check parameter ignore_columns_stock_lifetime_overrides in Settings-sheet)</t>
+  </si>
+  <si>
+    <t>stddev</t>
+  </si>
+  <si>
+    <t>shape</t>
+  </si>
+  <si>
+    <t>scale</t>
+  </si>
+  <si>
+    <t>condition</t>
+  </si>
+  <si>
+    <t>Landfill decay types</t>
+  </si>
+  <si>
+    <t>Wet</t>
+  </si>
+  <si>
+    <t>Dry</t>
+  </si>
+  <si>
+    <t>Managed</t>
+  </si>
+  <si>
+    <t>use_stock_lifetime_overrides</t>
+  </si>
+  <si>
+    <t>Use stock lifetime overrides</t>
+  </si>
+  <si>
+    <t>sheet_name_stock_lifetime_overrides</t>
+  </si>
+  <si>
+    <t>Stock lifetime overrides</t>
+  </si>
+  <si>
+    <t>ignore_columns_stock_lifetime_overrides</t>
+  </si>
+  <si>
+    <t>Ignore Excel columns defined in the list when reading data from stock lifetime overrides sheet. Each column name must be separated by comma (',')</t>
+  </si>
+  <si>
+    <t>skip_num_rows_stock_lifetime_overrides</t>
+  </si>
+  <si>
+    <t>Number of rows to skip when reading data for stock lifetime overrides (e.g. 2). NOTE: Header row must be the first row to read!</t>
+  </si>
+  <si>
+    <t>Name of the sheet that contains data for stock lifetime overrides</t>
+  </si>
+  <si>
+    <t>Name of the sheet that contains data for process positions in normalized format (position data in range [0,1])</t>
+  </si>
+  <si>
+    <t>Name of the sheet that contains data for transformation stage colors (e.g. Colors)</t>
+  </si>
+  <si>
+    <t>Name of the sheet that contains scenarios (flow variations)</t>
+  </si>
+  <si>
+    <t>Name of the sheet that contains data for Flows, (e.g. Flows)</t>
+  </si>
+  <si>
+    <t>Name of the sheet that contains data for Processes, e.g. (Processes)</t>
   </si>
 </sst>
 </file>
@@ -950,7 +1008,22 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="14">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCC0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <fill>
@@ -1407,7 +1480,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89FFA668-DA1A-459B-BD42-D0D7F7709F0D}">
-  <dimension ref="A2:E37"/>
+  <dimension ref="A2:E41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.7109375" bestFit="1" customWidth="1"/>
@@ -1424,12 +1497,12 @@
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B3" s="21" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C4" s="21"/>
       <c r="D4" s="21"/>
@@ -1443,7 +1516,7 @@
         <v>58</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>3</v>
@@ -1457,24 +1530,24 @@
         <v>1</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E7" t="s">
-        <v>68</v>
+        <v>239</v>
       </c>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="C8" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="D8" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E8" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.25">
@@ -1485,10 +1558,10 @@
         <v>2</v>
       </c>
       <c r="D9" s="22" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.25">
@@ -1499,24 +1572,24 @@
         <v>2</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E10" t="s">
-        <v>70</v>
+        <v>238</v>
       </c>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="C11" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="D11" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E11" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.25">
@@ -1527,413 +1600,489 @@
         <v>2</v>
       </c>
       <c r="D12" s="22" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E12" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C13" s="22">
         <v>2021</v>
       </c>
       <c r="D13" s="22" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E13" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C14" s="22">
         <v>2030</v>
       </c>
       <c r="D14" s="22" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E14" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C15" s="24" t="b">
         <v>0</v>
       </c>
       <c r="D15" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E15" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C16" s="24" t="b">
         <v>1</v>
       </c>
       <c r="D16" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E16" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C17" s="14">
         <v>0.1</v>
       </c>
       <c r="D17" s="22" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E17" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B18" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="C18" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="D18" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E18" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B19" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="C19" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D19" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E19" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B20" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C20" s="20">
         <v>-3.6666666666666701</v>
       </c>
       <c r="D20" s="20" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E20" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B21" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C21" s="24" t="b">
         <v>1</v>
       </c>
       <c r="D21" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E21" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B22" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C22" s="24" t="b">
         <v>1</v>
       </c>
       <c r="D22" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E22" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B23" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C23" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D23" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E23" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B24" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="C24" s="24" t="b">
         <v>1</v>
       </c>
       <c r="D24" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E24" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B25" t="s">
+        <v>195</v>
+      </c>
+      <c r="C25" t="s">
+        <v>197</v>
+      </c>
+      <c r="D25" t="s">
+        <v>92</v>
+      </c>
+      <c r="E25" t="s">
         <v>199</v>
-      </c>
-      <c r="C25" t="s">
-        <v>201</v>
-      </c>
-      <c r="D25" t="s">
-        <v>94</v>
-      </c>
-      <c r="E25" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B26" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C26" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D26" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E26" t="s">
-        <v>104</v>
+        <v>237</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B27" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="D27" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E27" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B28" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C28" s="24" t="b">
         <v>1</v>
       </c>
       <c r="D28" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E28" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B29" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C29" s="24" t="b">
         <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E29" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B30" t="s">
+        <v>123</v>
+      </c>
+      <c r="C30" t="s">
         <v>126</v>
       </c>
-      <c r="C30" t="s">
-        <v>129</v>
-      </c>
       <c r="D30" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E30" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B31" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C31" s="22" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="D31" s="22" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E31" t="s">
-        <v>148</v>
+        <v>236</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B32" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="D32" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E32" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B33" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="D33" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E33" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B34" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="D34" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E34" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B35" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="C35" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="D35" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E35" t="s">
-        <v>207</v>
+        <v>235</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B36" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="C36" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="D36" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E36" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B37" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="C37" s="24" t="b">
         <v>1</v>
       </c>
       <c r="D37" t="s">
+        <v>89</v>
+      </c>
+      <c r="E37" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>200</v>
+      </c>
+      <c r="B38" t="s">
+        <v>226</v>
+      </c>
+      <c r="C38" s="24" t="b">
+        <v>1</v>
+      </c>
+      <c r="D38" t="s">
+        <v>89</v>
+      </c>
+      <c r="E38" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>200</v>
+      </c>
+      <c r="B39" t="s">
+        <v>228</v>
+      </c>
+      <c r="C39" t="s">
+        <v>229</v>
+      </c>
+      <c r="D39" t="s">
         <v>91</v>
       </c>
-      <c r="E37" t="s">
-        <v>220</v>
+      <c r="E39" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>200</v>
+      </c>
+      <c r="B40" t="s">
+        <v>230</v>
+      </c>
+      <c r="C40" t="s">
+        <v>182</v>
+      </c>
+      <c r="D40" t="s">
+        <v>125</v>
+      </c>
+      <c r="E40" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>200</v>
+      </c>
+      <c r="B41" t="s">
+        <v>232</v>
+      </c>
+      <c r="C41">
+        <v>2</v>
+      </c>
+      <c r="D41" t="s">
+        <v>90</v>
+      </c>
+      <c r="E41" t="s">
+        <v>233</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="B6:E6" xr:uid="{89FFA668-DA1A-459B-BD42-D0D7F7709F0D}"/>
   <conditionalFormatting sqref="C15:C16">
+    <cfRule type="cellIs" dxfId="13" priority="11" operator="equal">
+      <formula>TRUE</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="12" priority="12" operator="notEqual">
+      <formula>TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C21:C22">
     <cfRule type="cellIs" dxfId="11" priority="9" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
@@ -1941,40 +2090,32 @@
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C21:C22">
-    <cfRule type="cellIs" dxfId="9" priority="7" operator="equal">
+  <conditionalFormatting sqref="C24">
+    <cfRule type="cellIs" dxfId="9" priority="5" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="8" operator="notEqual">
-      <formula>TRUE</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C24">
-    <cfRule type="cellIs" dxfId="7" priority="3" operator="equal">
-      <formula>TRUE</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="4" operator="notEqual">
+    <cfRule type="cellIs" dxfId="8" priority="6" operator="notEqual">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C28:C29">
-    <cfRule type="cellIs" dxfId="5" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="7" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="6" operator="notEqual">
+    <cfRule type="cellIs" dxfId="6" priority="8" operator="notEqual">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C37">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+  <conditionalFormatting sqref="C37:C38">
+    <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="notEqual">
+    <cfRule type="cellIs" dxfId="4" priority="4" operator="notEqual">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C15:C16 C21:C22 C28:C29 C24 C37" xr:uid="{79A7E31C-3284-4405-9B5F-03E099B07563}">
+  <dataValidations disablePrompts="1" count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C15:C16 C21:C22 C28:C29 C24 C37:C38" xr:uid="{79A7E31C-3284-4405-9B5F-03E099B07563}">
       <formula1>Boolean</formula1>
     </dataValidation>
   </dataValidations>
@@ -1982,7 +2123,7 @@
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="2">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{6A95900C-A9EB-48AB-A762-0F120DA62856}">
           <x14:formula1>
             <xm:f>'Data validation parameters'!$D$6:$D$9</xm:f>
@@ -2105,43 +2246,43 @@
     </row>
     <row r="3" spans="1:18" s="17" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="B3" s="16" t="s">
         <v>59</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="D3" s="16" t="s">
         <v>42</v>
       </c>
       <c r="E3" s="16" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="F3" s="16" t="s">
         <v>60</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="H3" s="16" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="I3" s="16" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="J3" s="16" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="K3" s="16" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="L3" s="16" t="s">
         <v>11</v>
       </c>
       <c r="M3" s="16" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="N3" s="16" t="s">
         <v>12</v>
@@ -2190,7 +2331,7 @@
         <v>0.34699999999999998</v>
       </c>
       <c r="R4" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" spans="1:18" ht="15.75" x14ac:dyDescent="0.3">
@@ -2224,7 +2365,7 @@
         <v>0.39200000000000002</v>
       </c>
       <c r="R5" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
@@ -2257,7 +2398,7 @@
         <v>0.05</v>
       </c>
       <c r="R6" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
@@ -2290,7 +2431,7 @@
         <v>0.53200000000000003</v>
       </c>
       <c r="R7" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="8" spans="1:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -2317,7 +2458,7 @@
         <v>38</v>
       </c>
       <c r="I8" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="P8">
         <v>0.752</v>
@@ -2326,7 +2467,7 @@
         <v>0.44400000000000001</v>
       </c>
       <c r="R8" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="9" spans="1:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -2353,7 +2494,7 @@
         <v>38</v>
       </c>
       <c r="I9" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="P9">
         <v>0.65600000000000003</v>
@@ -2362,7 +2503,7 @@
         <v>0.77300000000000002</v>
       </c>
       <c r="R9" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
@@ -2395,7 +2536,7 @@
         <v>0.9</v>
       </c>
       <c r="R10" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
@@ -2428,7 +2569,7 @@
         <v>0.16500000000000001</v>
       </c>
       <c r="R11" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
@@ -2461,7 +2602,7 @@
         <v>0.48299999999999998</v>
       </c>
       <c r="R12" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="18" ht="15.6" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2581,37 +2722,37 @@
       <c r="M2" s="2"/>
       <c r="N2" s="2"/>
       <c r="O2" s="2" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="P2" s="2"/>
     </row>
     <row r="3" spans="1:16" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="B3" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="H3" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="C3" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="D3" s="9" t="s">
+      <c r="I3" s="9" t="s">
         <v>170</v>
-      </c>
-      <c r="E3" s="9" t="s">
-        <v>171</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="G3" s="9" t="s">
-        <v>172</v>
-      </c>
-      <c r="H3" s="9" t="s">
-        <v>173</v>
-      </c>
-      <c r="I3" s="9" t="s">
-        <v>174</v>
       </c>
       <c r="J3" s="9" t="s">
         <v>58</v>
@@ -2623,13 +2764,13 @@
         <v>26</v>
       </c>
       <c r="M3" s="9" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="N3" s="10" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="O3" s="11" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="P3" s="12" t="s">
         <v>13</v>
@@ -3488,6 +3629,135 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD427C93-5971-4A1F-9BA5-0A112F61A8DE}">
+  <dimension ref="A1:J4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="37.85546875" customWidth="1"/>
+    <col min="2" max="2" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="35.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+    </row>
+    <row r="3" spans="1:10" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="I3" s="10" t="s">
+        <v>221</v>
+      </c>
+      <c r="J3" s="9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>205</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>2025</v>
+      </c>
+      <c r="E4">
+        <v>2030</v>
+      </c>
+      <c r="F4" s="3"/>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="NOTE" prompt="Used only in the following stock distribution types:_x000a_- Normal_x000a_- LogNormal_x000a_- FoldedNormal" sqref="F4" xr:uid="{EB58ED90-11CC-40D7-B560-63144E99B293}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="NOTE" prompt="Used only in the following stock distribution types:_x000a_- Weibull" sqref="G4:H4" xr:uid="{C2A4F33A-4C0F-44AA-B773-8DCE440EA2FB}"/>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="NOTE" prompt="Used only in the following stock distribution types:_x000a_- LandfillDecayWood_x000a_- LandfillDecayPaper" xr:uid="{23BA98F2-1DDD-4331-B721-E5AC9432C3B0}">
+          <x14:formula1>
+            <xm:f>'Data validation parameters'!$H$6:$H$9</xm:f>
+          </x14:formula1>
+          <xm:sqref>I4:I1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{715F83D3-09E8-436B-8662-E6CF9B40F02C}">
   <dimension ref="A1:D91"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3517,7 +3787,7 @@
         <v>2021</v>
       </c>
       <c r="B2" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="C2">
         <v>3.6999999999999998E-2</v>
@@ -3545,7 +3815,7 @@
         <v>2021</v>
       </c>
       <c r="B4" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="C4">
         <v>0.40899999999999997</v>
@@ -3573,7 +3843,7 @@
         <v>2021</v>
       </c>
       <c r="B6" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="C6">
         <v>0.752</v>
@@ -3587,7 +3857,7 @@
         <v>2021</v>
       </c>
       <c r="B7" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="C7">
         <v>0.65600000000000003</v>
@@ -3601,7 +3871,7 @@
         <v>2021</v>
       </c>
       <c r="B8" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="C8">
         <v>0.96599999999999997</v>
@@ -3615,7 +3885,7 @@
         <v>2021</v>
       </c>
       <c r="B9" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="C9">
         <v>0.69099999999999995</v>
@@ -3629,7 +3899,7 @@
         <v>2021</v>
       </c>
       <c r="B10" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="C10">
         <v>0.24299999999999999</v>
@@ -3643,7 +3913,7 @@
         <v>2022</v>
       </c>
       <c r="B11" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="C11">
         <v>3.6999999999999998E-2</v>
@@ -3671,7 +3941,7 @@
         <v>2022</v>
       </c>
       <c r="B13" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="C13">
         <v>0.40899999999999997</v>
@@ -3699,7 +3969,7 @@
         <v>2022</v>
       </c>
       <c r="B15" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="C15">
         <v>0.752</v>
@@ -3713,7 +3983,7 @@
         <v>2022</v>
       </c>
       <c r="B16" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="C16">
         <v>0.65600000000000003</v>
@@ -3727,7 +3997,7 @@
         <v>2022</v>
       </c>
       <c r="B17" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="C17">
         <v>0.96599999999999997</v>
@@ -3741,7 +4011,7 @@
         <v>2022</v>
       </c>
       <c r="B18" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="C18">
         <v>0.69099999999999995</v>
@@ -3755,7 +4025,7 @@
         <v>2022</v>
       </c>
       <c r="B19" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="C19">
         <v>0.24299999999999999</v>
@@ -3769,7 +4039,7 @@
         <v>2023</v>
       </c>
       <c r="B20" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="C20">
         <v>3.6999999999999998E-2</v>
@@ -3797,7 +4067,7 @@
         <v>2023</v>
       </c>
       <c r="B22" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="C22">
         <v>0.40899999999999997</v>
@@ -3825,7 +4095,7 @@
         <v>2023</v>
       </c>
       <c r="B24" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="C24">
         <v>0.752</v>
@@ -3839,7 +4109,7 @@
         <v>2023</v>
       </c>
       <c r="B25" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="C25">
         <v>0.65600000000000003</v>
@@ -3853,7 +4123,7 @@
         <v>2023</v>
       </c>
       <c r="B26" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="C26">
         <v>0.96599999999999997</v>
@@ -3867,7 +4137,7 @@
         <v>2023</v>
       </c>
       <c r="B27" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="C27">
         <v>0.69099999999999995</v>
@@ -3881,7 +4151,7 @@
         <v>2023</v>
       </c>
       <c r="B28" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="C28">
         <v>0.24299999999999999</v>
@@ -3895,7 +4165,7 @@
         <v>2024</v>
       </c>
       <c r="B29" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="C29">
         <v>3.6999999999999998E-2</v>
@@ -3923,7 +4193,7 @@
         <v>2024</v>
       </c>
       <c r="B31" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="C31">
         <v>0.40899999999999997</v>
@@ -3951,7 +4221,7 @@
         <v>2024</v>
       </c>
       <c r="B33" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="C33">
         <v>0.752</v>
@@ -3965,7 +4235,7 @@
         <v>2024</v>
       </c>
       <c r="B34" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="C34">
         <v>0.65600000000000003</v>
@@ -3979,7 +4249,7 @@
         <v>2024</v>
       </c>
       <c r="B35" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="C35">
         <v>0.96599999999999997</v>
@@ -3993,7 +4263,7 @@
         <v>2024</v>
       </c>
       <c r="B36" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="C36">
         <v>0.69099999999999995</v>
@@ -4007,7 +4277,7 @@
         <v>2024</v>
       </c>
       <c r="B37" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="C37">
         <v>0.24299999999999999</v>
@@ -4021,7 +4291,7 @@
         <v>2025</v>
       </c>
       <c r="B38" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="C38">
         <v>3.6999999999999998E-2</v>
@@ -4049,7 +4319,7 @@
         <v>2025</v>
       </c>
       <c r="B40" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="C40">
         <v>0.40899999999999997</v>
@@ -4077,7 +4347,7 @@
         <v>2025</v>
       </c>
       <c r="B42" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="C42">
         <v>0.752</v>
@@ -4091,7 +4361,7 @@
         <v>2025</v>
       </c>
       <c r="B43" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="C43">
         <v>0.65600000000000003</v>
@@ -4105,7 +4375,7 @@
         <v>2025</v>
       </c>
       <c r="B44" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="C44">
         <v>0.96599999999999997</v>
@@ -4119,7 +4389,7 @@
         <v>2025</v>
       </c>
       <c r="B45" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="C45">
         <v>0.69099999999999995</v>
@@ -4133,7 +4403,7 @@
         <v>2025</v>
       </c>
       <c r="B46" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="C46">
         <v>0.24299999999999999</v>
@@ -4147,7 +4417,7 @@
         <v>2026</v>
       </c>
       <c r="B47" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="C47">
         <v>3.6999999999999998E-2</v>
@@ -4175,7 +4445,7 @@
         <v>2026</v>
       </c>
       <c r="B49" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="C49">
         <v>0.40899999999999997</v>
@@ -4203,7 +4473,7 @@
         <v>2026</v>
       </c>
       <c r="B51" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="C51">
         <v>0.752</v>
@@ -4217,7 +4487,7 @@
         <v>2026</v>
       </c>
       <c r="B52" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="C52">
         <v>0.65600000000000003</v>
@@ -4231,7 +4501,7 @@
         <v>2026</v>
       </c>
       <c r="B53" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="C53">
         <v>0.96599999999999997</v>
@@ -4245,7 +4515,7 @@
         <v>2026</v>
       </c>
       <c r="B54" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="C54">
         <v>0.69099999999999995</v>
@@ -4259,7 +4529,7 @@
         <v>2026</v>
       </c>
       <c r="B55" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="C55">
         <v>0.24299999999999999</v>
@@ -4273,7 +4543,7 @@
         <v>2027</v>
       </c>
       <c r="B56" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="C56">
         <v>3.6999999999999998E-2</v>
@@ -4301,7 +4571,7 @@
         <v>2027</v>
       </c>
       <c r="B58" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="C58">
         <v>0.40899999999999997</v>
@@ -4329,7 +4599,7 @@
         <v>2027</v>
       </c>
       <c r="B60" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="C60">
         <v>0.752</v>
@@ -4343,7 +4613,7 @@
         <v>2027</v>
       </c>
       <c r="B61" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="C61">
         <v>0.65600000000000003</v>
@@ -4357,7 +4627,7 @@
         <v>2027</v>
       </c>
       <c r="B62" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="C62">
         <v>0.96599999999999997</v>
@@ -4371,7 +4641,7 @@
         <v>2027</v>
       </c>
       <c r="B63" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="C63">
         <v>0.69099999999999995</v>
@@ -4385,7 +4655,7 @@
         <v>2027</v>
       </c>
       <c r="B64" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="C64">
         <v>0.24299999999999999</v>
@@ -4399,7 +4669,7 @@
         <v>2028</v>
       </c>
       <c r="B65" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="C65">
         <v>3.6999999999999998E-2</v>
@@ -4427,7 +4697,7 @@
         <v>2028</v>
       </c>
       <c r="B67" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="C67">
         <v>0.40899999999999997</v>
@@ -4455,7 +4725,7 @@
         <v>2028</v>
       </c>
       <c r="B69" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="C69">
         <v>0.752</v>
@@ -4469,7 +4739,7 @@
         <v>2028</v>
       </c>
       <c r="B70" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="C70">
         <v>0.65600000000000003</v>
@@ -4483,7 +4753,7 @@
         <v>2028</v>
       </c>
       <c r="B71" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="C71">
         <v>0.96599999999999997</v>
@@ -4497,7 +4767,7 @@
         <v>2028</v>
       </c>
       <c r="B72" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="C72">
         <v>0.69099999999999995</v>
@@ -4511,7 +4781,7 @@
         <v>2028</v>
       </c>
       <c r="B73" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="C73">
         <v>0.24299999999999999</v>
@@ -4525,7 +4795,7 @@
         <v>2029</v>
       </c>
       <c r="B74" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="C74">
         <v>3.6999999999999998E-2</v>
@@ -4553,7 +4823,7 @@
         <v>2029</v>
       </c>
       <c r="B76" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="C76">
         <v>0.40899999999999997</v>
@@ -4581,7 +4851,7 @@
         <v>2029</v>
       </c>
       <c r="B78" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="C78">
         <v>0.752</v>
@@ -4595,7 +4865,7 @@
         <v>2029</v>
       </c>
       <c r="B79" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="C79">
         <v>0.65600000000000003</v>
@@ -4609,7 +4879,7 @@
         <v>2029</v>
       </c>
       <c r="B80" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="C80">
         <v>0.96599999999999997</v>
@@ -4623,7 +4893,7 @@
         <v>2029</v>
       </c>
       <c r="B81" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="C81">
         <v>0.69099999999999995</v>
@@ -4637,7 +4907,7 @@
         <v>2029</v>
       </c>
       <c r="B82" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="C82">
         <v>0.24299999999999999</v>
@@ -4651,7 +4921,7 @@
         <v>2030</v>
       </c>
       <c r="B83" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="C83">
         <v>3.6999999999999998E-2</v>
@@ -4679,7 +4949,7 @@
         <v>2030</v>
       </c>
       <c r="B85" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="C85">
         <v>0.40899999999999997</v>
@@ -4707,7 +4977,7 @@
         <v>2030</v>
       </c>
       <c r="B87" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="C87">
         <v>0.752</v>
@@ -4721,7 +4991,7 @@
         <v>2030</v>
       </c>
       <c r="B88" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="C88">
         <v>0.65600000000000003</v>
@@ -4735,7 +5005,7 @@
         <v>2030</v>
       </c>
       <c r="B89" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="C89">
         <v>0.96599999999999997</v>
@@ -4749,7 +5019,7 @@
         <v>2030</v>
       </c>
       <c r="B90" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="C90">
         <v>0.69099999999999995</v>
@@ -4763,7 +5033,7 @@
         <v>2030</v>
       </c>
       <c r="B91" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="C91">
         <v>0.24299999999999999</v>
@@ -4777,7 +5047,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43406F76-D4E1-4DE8-A811-C2AB881D41ED}">
   <dimension ref="A1:L3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4797,45 +5067,45 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="25" t="s">
+        <v>106</v>
+      </c>
+      <c r="B1" s="25" t="s">
+        <v>107</v>
+      </c>
+      <c r="C1" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="D1" s="25" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="25" t="s">
+      <c r="E1" s="25" t="s">
+        <v>187</v>
+      </c>
+      <c r="F1" s="25" t="s">
         <v>110</v>
       </c>
-      <c r="C1" s="25" t="s">
+      <c r="G1" s="25" t="s">
         <v>111</v>
       </c>
-      <c r="D1" s="25" t="s">
+      <c r="H1" s="25" t="s">
         <v>112</v>
       </c>
-      <c r="E1" s="25" t="s">
-        <v>191</v>
-      </c>
-      <c r="F1" s="25" t="s">
+      <c r="I1" s="25" t="s">
         <v>113</v>
       </c>
-      <c r="G1" s="25" t="s">
+      <c r="J1" s="25" t="s">
+        <v>210</v>
+      </c>
+      <c r="K1" s="25" t="s">
         <v>114</v>
       </c>
-      <c r="H1" s="25" t="s">
-        <v>115</v>
-      </c>
-      <c r="I1" s="25" t="s">
-        <v>116</v>
-      </c>
-      <c r="J1" s="25" t="s">
-        <v>215</v>
-      </c>
-      <c r="K1" s="25" t="s">
-        <v>117</v>
-      </c>
       <c r="L1" s="25" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>40</v>
@@ -4856,7 +5126,7 @@
         <v>2030</v>
       </c>
       <c r="I2" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="J2" s="24" t="b">
         <v>1</v>
@@ -4902,7 +5172,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA92C4F1-884F-4740-8793-4A0AB47EED3D}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4913,10 +5183,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -4924,7 +5194,7 @@
         <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -4932,7 +5202,7 @@
         <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -4940,7 +5210,7 @@
         <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -4948,7 +5218,7 @@
         <v>37</v>
       </c>
       <c r="B5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -4956,7 +5226,7 @@
         <v>17</v>
       </c>
       <c r="B6" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -4964,7 +5234,7 @@
         <v>35</v>
       </c>
       <c r="B7" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -4972,18 +5242,18 @@
         <v>36</v>
       </c>
       <c r="B8" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B9" t="s">
+        <v>145</v>
+      </c>
+      <c r="C9" t="s">
         <v>149</v>
-      </c>
-      <c r="C9" t="s">
-        <v>153</v>
       </c>
     </row>
   </sheetData>
@@ -4992,9 +5262,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C12935D7-39CC-4336-870D-98DAC14A69ED}">
-  <dimension ref="B2:G13"/>
+  <dimension ref="B2:H13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
@@ -5003,40 +5273,44 @@
     <col min="5" max="5" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.42578125" customWidth="1"/>
     <col min="11" max="11" width="30.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="18" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G5" s="18" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
+        <v>196</v>
+      </c>
+      <c r="H5" s="18" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>54</v>
       </c>
@@ -5044,19 +5318,22 @@
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="E6" t="s">
         <v>58</v>
       </c>
       <c r="F6" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G6" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+        <v>197</v>
+      </c>
+      <c r="H6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>38</v>
       </c>
@@ -5064,58 +5341,64 @@
         <v>0</v>
       </c>
       <c r="D7" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="E7" t="s">
         <v>9</v>
       </c>
       <c r="F7" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G7" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
+        <v>198</v>
+      </c>
+      <c r="H7" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>55</v>
       </c>
       <c r="D8" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F8" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+      <c r="H8" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>57</v>
       </c>
       <c r="D9" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F9" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -5125,27 +5408,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7536dd80-7d39-48e8-9ae3-b4166f580a2d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="145cc194-9bea-4db6-b116-a042a4529fcd" xsi:nil="true"/>
-    <Comment xmlns="7536dd80-7d39-48e8-9ae3-b4166f580a2d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Asiakirja" ma:contentTypeID="0x010100806C55B750152A459818B636E97A41C3" ma:contentTypeVersion="19" ma:contentTypeDescription="Luo uusi asiakirja." ma:contentTypeScope="" ma:versionID="74fd9cb75cef04cf26a1ff9ddef01b4b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7536dd80-7d39-48e8-9ae3-b4166f580a2d" xmlns:ns3="145cc194-9bea-4db6-b116-a042a4529fcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="afbcbfdd38894bc2ff0644b00c8ec680" ns2:_="" ns3:_="">
     <xsd:import namespace="7536dd80-7d39-48e8-9ae3-b4166f580a2d"/>
@@ -5408,10 +5670,42 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7536dd80-7d39-48e8-9ae3-b4166f580a2d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="145cc194-9bea-4db6-b116-a042a4529fcd" xsi:nil="true"/>
+    <Comment xmlns="7536dd80-7d39-48e8-9ae3-b4166f580a2d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AB3C6F0-DB35-46F0-8FEB-B5E57B48A727}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D60021C7-CA75-4673-96EA-55284BF81134}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="7536dd80-7d39-48e8-9ae3-b4166f580a2d"/>
+    <ds:schemaRef ds:uri="145cc194-9bea-4db6-b116-a042a4529fcd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -5434,20 +5728,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D60021C7-CA75-4673-96EA-55284BF81134}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AB3C6F0-DB35-46F0-8FEB-B5E57B48A727}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="7536dd80-7d39-48e8-9ae3-b4166f580a2d"/>
-    <ds:schemaRef ds:uri="145cc194-9bea-4db6-b116-a042a4529fcd"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Emptied stock lifetime override sheet in example_scenario.xlsx
</commit_message>
<xml_diff>
--- a/src/aiphoria/data/example_scenario.xlsx
+++ b/src/aiphoria/data/example_scenario.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\PythonProjects\aiphoria\src\aiphoria\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FF67D8E-CB75-437F-A89D-3471ED78FF46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BB4364F-BEE6-468C-9CE3-4010F84BFE50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{1000A452-A98F-45C1-B843-91F7F67E097C}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="240">
   <si>
     <t>Years</t>
   </si>
@@ -1008,22 +1008,7 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="14">
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCC0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="12">
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <fill>
@@ -2075,42 +2060,42 @@
   </sheetData>
   <autoFilter ref="B6:E6" xr:uid="{89FFA668-DA1A-459B-BD42-D0D7F7709F0D}"/>
   <conditionalFormatting sqref="C15:C16">
-    <cfRule type="cellIs" dxfId="13" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="11" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="12" operator="notEqual">
+    <cfRule type="cellIs" dxfId="10" priority="12" operator="notEqual">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C21:C22">
-    <cfRule type="cellIs" dxfId="11" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="9" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="10" operator="notEqual">
+    <cfRule type="cellIs" dxfId="8" priority="10" operator="notEqual">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C24">
-    <cfRule type="cellIs" dxfId="9" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="5" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="6" operator="notEqual">
+    <cfRule type="cellIs" dxfId="6" priority="6" operator="notEqual">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C28:C29">
-    <cfRule type="cellIs" dxfId="7" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="7" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="8" operator="notEqual">
+    <cfRule type="cellIs" dxfId="4" priority="8" operator="notEqual">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C37:C38">
-    <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="4" operator="notEqual">
+    <cfRule type="cellIs" dxfId="2" priority="4" operator="notEqual">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3722,18 +3707,6 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
-        <v>205</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4">
-        <v>2025</v>
-      </c>
-      <c r="E4">
-        <v>2030</v>
-      </c>
       <c r="F4" s="3"/>
     </row>
   </sheetData>
@@ -5138,10 +5111,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="J2">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="notEqual">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="notEqual">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5671,6 +5644,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="7536dd80-7d39-48e8-9ae3-b4166f580a2d">
@@ -5680,15 +5662,6 @@
     <Comment xmlns="7536dd80-7d39-48e8-9ae3-b4166f580a2d" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5711,6 +5684,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AB3C6F0-DB35-46F0-8FEB-B5E57B48A727}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{557FAA9C-B184-448F-B58D-00E4D46BDD72}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -5725,12 +5706,4 @@
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AB3C6F0-DB35-46F0-8FEB-B5E57B48A727}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Added shields to README.md and added data validation to column headers in example_scenario.xlsx
</commit_message>
<xml_diff>
--- a/src/aiphoria/data/example_scenario.xlsx
+++ b/src/aiphoria/data/example_scenario.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\PythonProjects\aiphoria\src\aiphoria\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BB4364F-BEE6-468C-9CE3-4010F84BFE50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09A8A7FA-C9CB-45DD-8B36-E2AF8C325E31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{1000A452-A98F-45C1-B843-91F7F67E097C}"/>
+    <workbookView xWindow="3120" yWindow="2130" windowWidth="24060" windowHeight="12480" xr2:uid="{1000A452-A98F-45C1-B843-91F7F67E097C}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="11" r:id="rId1"/>
@@ -2099,7 +2099,7 @@
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C15:C16 C21:C22 C28:C29 C24 C37:C38" xr:uid="{79A7E31C-3284-4405-9B5F-03E099B07563}">
       <formula1>Boolean</formula1>
     </dataValidation>
@@ -2108,7 +2108,7 @@
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="2">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{6A95900C-A9EB-48AB-A762-0F120DA62856}">
           <x14:formula1>
             <xm:f>'Data validation parameters'!$D$6:$D$9</xm:f>
@@ -3710,19 +3710,20 @@
       <c r="F4" s="3"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="NOTE" prompt="Used only in the following stock distribution types:_x000a_- Normal_x000a_- LogNormal_x000a_- FoldedNormal" sqref="F4" xr:uid="{EB58ED90-11CC-40D7-B560-63144E99B293}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="NOTE" prompt="Used only in the following stock distribution types:_x000a_- Weibull" sqref="G4:H4" xr:uid="{C2A4F33A-4C0F-44AA-B773-8DCE440EA2FB}"/>
+  <dataValidations xWindow="985" yWindow="379" count="3">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="NOTE" prompt="Used only in the following stock distribution types:_x000a_- Normal_x000a_- LogNormal_x000a_- FoldedNormal" sqref="F4:F1048576 F3" xr:uid="{EB58ED90-11CC-40D7-B560-63144E99B293}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="NOTE" prompt="Used only in the following stock distribution types:_x000a_- Weibull" sqref="G3:G1048576 H3:H4 H6:H1048576 H5" xr:uid="{C2A4F33A-4C0F-44AA-B773-8DCE440EA2FB}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="NOTE" prompt="Used only in the following stock distribution types:_x000a_- LandfillDecayWood_x000a_- LandfillDecayPaper" sqref="I3" xr:uid="{9247F767-8020-484B-8E5F-041BF9D0E8CE}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xWindow="985" yWindow="379" count="1">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="NOTE" prompt="Used only in the following stock distribution types:_x000a_- LandfillDecayWood_x000a_- LandfillDecayPaper" xr:uid="{23BA98F2-1DDD-4331-B721-E5AC9432C3B0}">
           <x14:formula1>
             <xm:f>'Data validation parameters'!$H$6:$H$9</xm:f>
           </x14:formula1>
-          <xm:sqref>I4:I1048576</xm:sqref>
+          <xm:sqref>I5:I1048576 I4</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -5644,15 +5645,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="7536dd80-7d39-48e8-9ae3-b4166f580a2d">
@@ -5662,6 +5654,15 @@
     <Comment xmlns="7536dd80-7d39-48e8-9ae3-b4166f580a2d" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5684,14 +5685,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AB3C6F0-DB35-46F0-8FEB-B5E57B48A727}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{557FAA9C-B184-448F-B58D-00E4D46BDD72}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -5706,4 +5699,12 @@
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AB3C6F0-DB35-46F0-8FEB-B5E57B48A727}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
- Fixed typo in parameter in example scenario file - Added unit tests and integration tests - Added new parameter "parameter_overrides" for run_scenarios() to allow changing parameters outside settings file - Added new parameter "parameter_overrides" to run_example() to allow changing parameters outside settings file - Omit ODYM files from coverage tests - Added pytest parameters to pyproject.toml
</commit_message>
<xml_diff>
--- a/src/aiphoria/data/example_scenario.xlsx
+++ b/src/aiphoria/data/example_scenario.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\PythonProjects\aiphoria\src\aiphoria\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09A8A7FA-C9CB-45DD-8B36-E2AF8C325E31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4739C9D-770B-4127-A07F-F56B69885A29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="2130" windowWidth="24060" windowHeight="12480" xr2:uid="{1000A452-A98F-45C1-B843-91F7F67E097C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{1000A452-A98F-45C1-B843-91F7F67E097C}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="11" r:id="rId1"/>
@@ -677,9 +677,6 @@
     <t>LandfillDecayPaper</t>
   </si>
   <si>
-    <t>prioritize_transformation_stage</t>
-  </si>
-  <si>
     <t>scenario_type</t>
   </si>
   <si>
@@ -813,6 +810,9 @@
   </si>
   <si>
     <t>Name of the sheet that contains data for Processes, e.g. (Processes)</t>
+  </si>
+  <si>
+    <t>prioritize_transformation_stages</t>
   </si>
 </sst>
 </file>
@@ -1518,7 +1518,7 @@
         <v>92</v>
       </c>
       <c r="E7" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.25">
@@ -1560,7 +1560,7 @@
         <v>91</v>
       </c>
       <c r="E10" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.25">
@@ -1663,7 +1663,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B18" t="s">
         <v>173</v>
@@ -1680,7 +1680,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B19" t="s">
         <v>174</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B20" t="s">
         <v>77</v>
@@ -1714,7 +1714,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B21" t="s">
         <v>87</v>
@@ -1731,7 +1731,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B22" t="s">
         <v>86</v>
@@ -1748,7 +1748,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B23" t="s">
         <v>94</v>
@@ -1765,7 +1765,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B24" t="s">
         <v>185</v>
@@ -1782,24 +1782,24 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B25" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C25" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D25" t="s">
         <v>92</v>
       </c>
       <c r="E25" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B26" t="s">
         <v>100</v>
@@ -1811,12 +1811,12 @@
         <v>91</v>
       </c>
       <c r="E26" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B27" t="s">
         <v>161</v>
@@ -1830,7 +1830,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B28" t="s">
         <v>102</v>
@@ -1847,7 +1847,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B29" t="s">
         <v>104</v>
@@ -1864,7 +1864,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B30" t="s">
         <v>123</v>
@@ -1881,7 +1881,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B31" t="s">
         <v>143</v>
@@ -1893,12 +1893,12 @@
         <v>91</v>
       </c>
       <c r="E31" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B32" t="s">
         <v>162</v>
@@ -1912,7 +1912,7 @@
     </row>
     <row r="33" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B33" t="s">
         <v>188</v>
@@ -1926,10 +1926,10 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B34" t="s">
-        <v>194</v>
+        <v>239</v>
       </c>
       <c r="D34" t="s">
         <v>125</v>
@@ -1940,44 +1940,44 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>199</v>
+      </c>
+      <c r="B35" t="s">
         <v>200</v>
       </c>
-      <c r="B35" t="s">
+      <c r="C35" t="s">
         <v>201</v>
-      </c>
-      <c r="C35" t="s">
-        <v>202</v>
       </c>
       <c r="D35" t="s">
         <v>91</v>
       </c>
       <c r="E35" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B36" t="s">
+        <v>210</v>
+      </c>
+      <c r="C36" t="s">
         <v>211</v>
-      </c>
-      <c r="C36" t="s">
-        <v>212</v>
       </c>
       <c r="D36" t="s">
         <v>91</v>
       </c>
       <c r="E36" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B37" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C37" s="24" t="b">
         <v>1</v>
@@ -1986,15 +1986,15 @@
         <v>89</v>
       </c>
       <c r="E37" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B38" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C38" s="24" t="b">
         <v>1</v>
@@ -2003,32 +2003,32 @@
         <v>89</v>
       </c>
       <c r="E38" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B39" t="s">
+        <v>227</v>
+      </c>
+      <c r="C39" t="s">
         <v>228</v>
-      </c>
-      <c r="C39" t="s">
-        <v>229</v>
       </c>
       <c r="D39" t="s">
         <v>91</v>
       </c>
       <c r="E39" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B40" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C40" t="s">
         <v>182</v>
@@ -2037,15 +2037,15 @@
         <v>125</v>
       </c>
       <c r="E40" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B41" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C41">
         <v>2</v>
@@ -2054,7 +2054,7 @@
         <v>90</v>
       </c>
       <c r="E41" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
   </sheetData>
@@ -3645,13 +3645,13 @@
         <v>5</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="I1" s="2" t="s">
         <v>5</v>
@@ -3676,7 +3676,7 @@
     </row>
     <row r="3" spans="1:10" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>42</v>
@@ -3691,16 +3691,16 @@
         <v>112</v>
       </c>
       <c r="F3" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="G3" s="9" t="s">
         <v>218</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="H3" s="9" t="s">
         <v>219</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="I3" s="10" t="s">
         <v>220</v>
-      </c>
-      <c r="I3" s="10" t="s">
-        <v>221</v>
       </c>
       <c r="J3" s="9" t="s">
         <v>13</v>
@@ -3761,7 +3761,7 @@
         <v>2021</v>
       </c>
       <c r="B2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C2">
         <v>3.6999999999999998E-2</v>
@@ -3789,7 +3789,7 @@
         <v>2021</v>
       </c>
       <c r="B4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C4">
         <v>0.40899999999999997</v>
@@ -3817,7 +3817,7 @@
         <v>2021</v>
       </c>
       <c r="B6" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C6">
         <v>0.752</v>
@@ -3831,7 +3831,7 @@
         <v>2021</v>
       </c>
       <c r="B7" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C7">
         <v>0.65600000000000003</v>
@@ -3845,7 +3845,7 @@
         <v>2021</v>
       </c>
       <c r="B8" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C8">
         <v>0.96599999999999997</v>
@@ -3859,7 +3859,7 @@
         <v>2021</v>
       </c>
       <c r="B9" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C9">
         <v>0.69099999999999995</v>
@@ -3873,7 +3873,7 @@
         <v>2021</v>
       </c>
       <c r="B10" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C10">
         <v>0.24299999999999999</v>
@@ -3887,7 +3887,7 @@
         <v>2022</v>
       </c>
       <c r="B11" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C11">
         <v>3.6999999999999998E-2</v>
@@ -3915,7 +3915,7 @@
         <v>2022</v>
       </c>
       <c r="B13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C13">
         <v>0.40899999999999997</v>
@@ -3943,7 +3943,7 @@
         <v>2022</v>
       </c>
       <c r="B15" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C15">
         <v>0.752</v>
@@ -3957,7 +3957,7 @@
         <v>2022</v>
       </c>
       <c r="B16" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C16">
         <v>0.65600000000000003</v>
@@ -3971,7 +3971,7 @@
         <v>2022</v>
       </c>
       <c r="B17" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C17">
         <v>0.96599999999999997</v>
@@ -3985,7 +3985,7 @@
         <v>2022</v>
       </c>
       <c r="B18" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C18">
         <v>0.69099999999999995</v>
@@ -3999,7 +3999,7 @@
         <v>2022</v>
       </c>
       <c r="B19" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C19">
         <v>0.24299999999999999</v>
@@ -4013,7 +4013,7 @@
         <v>2023</v>
       </c>
       <c r="B20" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C20">
         <v>3.6999999999999998E-2</v>
@@ -4041,7 +4041,7 @@
         <v>2023</v>
       </c>
       <c r="B22" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C22">
         <v>0.40899999999999997</v>
@@ -4069,7 +4069,7 @@
         <v>2023</v>
       </c>
       <c r="B24" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C24">
         <v>0.752</v>
@@ -4083,7 +4083,7 @@
         <v>2023</v>
       </c>
       <c r="B25" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C25">
         <v>0.65600000000000003</v>
@@ -4097,7 +4097,7 @@
         <v>2023</v>
       </c>
       <c r="B26" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C26">
         <v>0.96599999999999997</v>
@@ -4111,7 +4111,7 @@
         <v>2023</v>
       </c>
       <c r="B27" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C27">
         <v>0.69099999999999995</v>
@@ -4125,7 +4125,7 @@
         <v>2023</v>
       </c>
       <c r="B28" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C28">
         <v>0.24299999999999999</v>
@@ -4139,7 +4139,7 @@
         <v>2024</v>
       </c>
       <c r="B29" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C29">
         <v>3.6999999999999998E-2</v>
@@ -4167,7 +4167,7 @@
         <v>2024</v>
       </c>
       <c r="B31" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C31">
         <v>0.40899999999999997</v>
@@ -4195,7 +4195,7 @@
         <v>2024</v>
       </c>
       <c r="B33" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C33">
         <v>0.752</v>
@@ -4209,7 +4209,7 @@
         <v>2024</v>
       </c>
       <c r="B34" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C34">
         <v>0.65600000000000003</v>
@@ -4223,7 +4223,7 @@
         <v>2024</v>
       </c>
       <c r="B35" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C35">
         <v>0.96599999999999997</v>
@@ -4237,7 +4237,7 @@
         <v>2024</v>
       </c>
       <c r="B36" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C36">
         <v>0.69099999999999995</v>
@@ -4251,7 +4251,7 @@
         <v>2024</v>
       </c>
       <c r="B37" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C37">
         <v>0.24299999999999999</v>
@@ -4265,7 +4265,7 @@
         <v>2025</v>
       </c>
       <c r="B38" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C38">
         <v>3.6999999999999998E-2</v>
@@ -4293,7 +4293,7 @@
         <v>2025</v>
       </c>
       <c r="B40" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C40">
         <v>0.40899999999999997</v>
@@ -4321,7 +4321,7 @@
         <v>2025</v>
       </c>
       <c r="B42" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C42">
         <v>0.752</v>
@@ -4335,7 +4335,7 @@
         <v>2025</v>
       </c>
       <c r="B43" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C43">
         <v>0.65600000000000003</v>
@@ -4349,7 +4349,7 @@
         <v>2025</v>
       </c>
       <c r="B44" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C44">
         <v>0.96599999999999997</v>
@@ -4363,7 +4363,7 @@
         <v>2025</v>
       </c>
       <c r="B45" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C45">
         <v>0.69099999999999995</v>
@@ -4377,7 +4377,7 @@
         <v>2025</v>
       </c>
       <c r="B46" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C46">
         <v>0.24299999999999999</v>
@@ -4391,7 +4391,7 @@
         <v>2026</v>
       </c>
       <c r="B47" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C47">
         <v>3.6999999999999998E-2</v>
@@ -4419,7 +4419,7 @@
         <v>2026</v>
       </c>
       <c r="B49" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C49">
         <v>0.40899999999999997</v>
@@ -4447,7 +4447,7 @@
         <v>2026</v>
       </c>
       <c r="B51" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C51">
         <v>0.752</v>
@@ -4461,7 +4461,7 @@
         <v>2026</v>
       </c>
       <c r="B52" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C52">
         <v>0.65600000000000003</v>
@@ -4475,7 +4475,7 @@
         <v>2026</v>
       </c>
       <c r="B53" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C53">
         <v>0.96599999999999997</v>
@@ -4489,7 +4489,7 @@
         <v>2026</v>
       </c>
       <c r="B54" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C54">
         <v>0.69099999999999995</v>
@@ -4503,7 +4503,7 @@
         <v>2026</v>
       </c>
       <c r="B55" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C55">
         <v>0.24299999999999999</v>
@@ -4517,7 +4517,7 @@
         <v>2027</v>
       </c>
       <c r="B56" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C56">
         <v>3.6999999999999998E-2</v>
@@ -4545,7 +4545,7 @@
         <v>2027</v>
       </c>
       <c r="B58" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C58">
         <v>0.40899999999999997</v>
@@ -4573,7 +4573,7 @@
         <v>2027</v>
       </c>
       <c r="B60" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C60">
         <v>0.752</v>
@@ -4587,7 +4587,7 @@
         <v>2027</v>
       </c>
       <c r="B61" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C61">
         <v>0.65600000000000003</v>
@@ -4601,7 +4601,7 @@
         <v>2027</v>
       </c>
       <c r="B62" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C62">
         <v>0.96599999999999997</v>
@@ -4615,7 +4615,7 @@
         <v>2027</v>
       </c>
       <c r="B63" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C63">
         <v>0.69099999999999995</v>
@@ -4629,7 +4629,7 @@
         <v>2027</v>
       </c>
       <c r="B64" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C64">
         <v>0.24299999999999999</v>
@@ -4643,7 +4643,7 @@
         <v>2028</v>
       </c>
       <c r="B65" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C65">
         <v>3.6999999999999998E-2</v>
@@ -4671,7 +4671,7 @@
         <v>2028</v>
       </c>
       <c r="B67" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C67">
         <v>0.40899999999999997</v>
@@ -4699,7 +4699,7 @@
         <v>2028</v>
       </c>
       <c r="B69" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C69">
         <v>0.752</v>
@@ -4713,7 +4713,7 @@
         <v>2028</v>
       </c>
       <c r="B70" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C70">
         <v>0.65600000000000003</v>
@@ -4727,7 +4727,7 @@
         <v>2028</v>
       </c>
       <c r="B71" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C71">
         <v>0.96599999999999997</v>
@@ -4741,7 +4741,7 @@
         <v>2028</v>
       </c>
       <c r="B72" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C72">
         <v>0.69099999999999995</v>
@@ -4755,7 +4755,7 @@
         <v>2028</v>
       </c>
       <c r="B73" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C73">
         <v>0.24299999999999999</v>
@@ -4769,7 +4769,7 @@
         <v>2029</v>
       </c>
       <c r="B74" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C74">
         <v>3.6999999999999998E-2</v>
@@ -4797,7 +4797,7 @@
         <v>2029</v>
       </c>
       <c r="B76" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C76">
         <v>0.40899999999999997</v>
@@ -4825,7 +4825,7 @@
         <v>2029</v>
       </c>
       <c r="B78" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C78">
         <v>0.752</v>
@@ -4839,7 +4839,7 @@
         <v>2029</v>
       </c>
       <c r="B79" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C79">
         <v>0.65600000000000003</v>
@@ -4853,7 +4853,7 @@
         <v>2029</v>
       </c>
       <c r="B80" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C80">
         <v>0.96599999999999997</v>
@@ -4867,7 +4867,7 @@
         <v>2029</v>
       </c>
       <c r="B81" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C81">
         <v>0.69099999999999995</v>
@@ -4881,7 +4881,7 @@
         <v>2029</v>
       </c>
       <c r="B82" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C82">
         <v>0.24299999999999999</v>
@@ -4895,7 +4895,7 @@
         <v>2030</v>
       </c>
       <c r="B83" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C83">
         <v>3.6999999999999998E-2</v>
@@ -4923,7 +4923,7 @@
         <v>2030</v>
       </c>
       <c r="B85" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C85">
         <v>0.40899999999999997</v>
@@ -4951,7 +4951,7 @@
         <v>2030</v>
       </c>
       <c r="B87" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C87">
         <v>0.752</v>
@@ -4965,7 +4965,7 @@
         <v>2030</v>
       </c>
       <c r="B88" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C88">
         <v>0.65600000000000003</v>
@@ -4979,7 +4979,7 @@
         <v>2030</v>
       </c>
       <c r="B89" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C89">
         <v>0.96599999999999997</v>
@@ -4993,7 +4993,7 @@
         <v>2030</v>
       </c>
       <c r="B90" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C90">
         <v>0.69099999999999995</v>
@@ -5007,7 +5007,7 @@
         <v>2030</v>
       </c>
       <c r="B91" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C91">
         <v>0.24299999999999999</v>
@@ -5068,7 +5068,7 @@
         <v>113</v>
       </c>
       <c r="J1" s="25" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="K1" s="25" t="s">
         <v>114</v>
@@ -5278,10 +5278,10 @@
         <v>113</v>
       </c>
       <c r="G5" s="18" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="H5" s="18" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.25">
@@ -5301,10 +5301,10 @@
         <v>119</v>
       </c>
       <c r="G6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="H6" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.25">
@@ -5324,10 +5324,10 @@
         <v>120</v>
       </c>
       <c r="G7" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="H7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
@@ -5341,7 +5341,7 @@
         <v>121</v>
       </c>
       <c r="H8" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated: - FlowModifierSolver captures relative flow errors better with more detailed error messages Added: - New input files for tests
</commit_message>
<xml_diff>
--- a/src/aiphoria/data/example_scenario.xlsx
+++ b/src/aiphoria/data/example_scenario.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\PythonProjects\aiphoria\src\aiphoria\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4739C9D-770B-4127-A07F-F56B69885A29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B89CE2A-CFA9-4264-9CC9-BBBA7361EB5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{1000A452-A98F-45C1-B843-91F7F67E097C}"/>
+    <workbookView xWindow="-25635" yWindow="2265" windowWidth="21600" windowHeight="11295" activeTab="5" xr2:uid="{1000A452-A98F-45C1-B843-91F7F67E097C}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="11" r:id="rId1"/>
@@ -5382,6 +5382,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Asiakirja" ma:contentTypeID="0x010100806C55B750152A459818B636E97A41C3" ma:contentTypeVersion="19" ma:contentTypeDescription="Luo uusi asiakirja." ma:contentTypeScope="" ma:versionID="74fd9cb75cef04cf26a1ff9ddef01b4b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7536dd80-7d39-48e8-9ae3-b4166f580a2d" xmlns:ns3="145cc194-9bea-4db6-b116-a042a4529fcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="afbcbfdd38894bc2ff0644b00c8ec680" ns2:_="" ns3:_="">
     <xsd:import namespace="7536dd80-7d39-48e8-9ae3-b4166f580a2d"/>
@@ -5644,7 +5653,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="7536dd80-7d39-48e8-9ae3-b4166f580a2d">
@@ -5656,16 +5665,15 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AB3C6F0-DB35-46F0-8FEB-B5E57B48A727}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D60021C7-CA75-4673-96EA-55284BF81134}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5684,7 +5692,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{557FAA9C-B184-448F-B58D-00E4D46BDD72}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -5699,12 +5707,4 @@
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AB3C6F0-DB35-46F0-8FEB-B5E57B48A727}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>